<commit_message>
Final Changes, This is to be submitted
</commit_message>
<xml_diff>
--- a/CST1500_Contribution_Spreadsheet.xlsx
+++ b/CST1500_Contribution_Spreadsheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E923F7BD-3328-4C95-9F9E-36F94B35D2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{566B5447-A6F5-43C0-8282-0D662EB61BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="X4ZlR6JvWvWiB8zDukt5NYZ+6LUTy5vldl3/puEK4WeKo43ORe1O7rqBGokIeM8B6uDTq5MPEFA8n6QMvQb6Ng==" workbookSaltValue="6cw7hsiy8i7NdCSQb2xZ6Q==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -621,10 +621,10 @@
       </c>
       <c r="D8" s="12"/>
       <c r="E8" s="8">
+        <v>0</v>
+      </c>
+      <c r="F8" s="8">
         <v>1</v>
-      </c>
-      <c r="F8" s="8">
-        <v>0</v>
       </c>
       <c r="G8" s="8">
         <v>0</v>
@@ -647,10 +647,10 @@
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="8">
         <v>0</v>
@@ -699,12 +699,15 @@
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="14">
+        <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="F11" s="14">
+        <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="G11" s="14">
+        <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="H11" t="str">
@@ -725,13 +728,16 @@
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="8">
-        <v>0.5</v>
+        <f>1/3</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="F12" s="8">
-        <v>0</v>
+        <f>1/3</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="G12" s="8">
-        <v>0.5</v>
+        <f>1/3</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="0"/>
@@ -1215,6 +1221,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="13086975-c1d0-4a06-9c64-3fd990a1352b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B5E4D76328569F43B69913F006A221B2" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="56a22f8d817eb20ed3693209c2a5d799">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="13086975-c1d0-4a06-9c64-3fd990a1352b" xmlns:ns4="f8d07fca-19e9-492a-8c2e-699b0725e001" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cc6f122d176e53dc02b49ce47b3b9659" ns3:_="" ns4:_="">
     <xsd:import namespace="13086975-c1d0-4a06-9c64-3fd990a1352b"/>
@@ -1467,24 +1490,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA851950-2E95-4230-BEB3-A25E4F3EE837}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="f8d07fca-19e9-492a-8c2e-699b0725e001"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="13086975-c1d0-4a06-9c64-3fd990a1352b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="13086975-c1d0-4a06-9c64-3fd990a1352b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCA5D7B-7CC0-427F-B0CE-DC2F534D9F7A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85932C06-FB31-498A-8232-D2B799F2D6AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1501,29 +1532,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCCA5D7B-7CC0-427F-B0CE-DC2F534D9F7A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA851950-2E95-4230-BEB3-A25E4F3EE837}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="f8d07fca-19e9-492a-8c2e-699b0725e001"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="13086975-c1d0-4a06-9c64-3fd990a1352b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>